<commit_message>
Update responsive design and deployment docs
</commit_message>
<xml_diff>
--- a/data/earthwork.xlsx
+++ b/data/earthwork.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\titiw\Desktop\Dashboard เว็บไซต์สำหรับงาน Earthwork\earthwork_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B90CAC-E36D-4978-8292-3F683E9C9402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5F20D6-70B2-447C-9152-9FFA626CCA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -731,8 +731,8 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.125" customWidth="1"/>
-    <col min="2" max="2" width="16.375" customWidth="1"/>
+    <col min="1" max="1" width="38.5" customWidth="1"/>
+    <col min="2" max="2" width="18.625" customWidth="1"/>
     <col min="3" max="3" width="18.5" customWidth="1"/>
     <col min="4" max="4" width="19.375" customWidth="1"/>
     <col min="5" max="5" width="19.25" customWidth="1"/>

</xml_diff>